<commit_message>
Rename Name and Property of JSON data.
</commit_message>
<xml_diff>
--- a/JSON Whole Model/ASTIDC-STAN-HE-EPD-MVB1-M-E-0002_name_table.xlsx
+++ b/JSON Whole Model/ASTIDC-STAN-HE-EPD-MVB1-M-E-0002_name_table.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1JNL9322340_A-1JNL9322340 - Pyramid</t>
+          <t>A-1JNL9322340 - Pyramid</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -471,33 +471,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1JNL9362899_A-Electrical design requirements, MVS1, NER, Aux Tx-building, Cable ways</t>
+          <t>A-Cable Ladder 90 450</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cd06ec2a-dde8-35e7-bb84-94eaba646aaa</t>
+          <t>c9232a6d-75c5-3739-a3c2-3777ac67e597</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1JNL9441111_A-Cable Ladder 90 450</t>
+          <t>A-Cable Ladder 90 450</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>c9232a6d-75c5-3739-a3c2-3777ac67e597</t>
+          <t>3d931300-8be8-3a23-a464-9cedb7d98460</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -507,15 +507,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1JNL9441111_A-Cable Ladder 90 450</t>
+          <t>A-Cable Ladder 90 450</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3d931300-8be8-3a23-a464-9cedb7d98460</t>
+          <t>19f22aef-af24-3a1c-b63f-1703e94e50ba</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -525,115 +525,115 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1JNL9441111_A-Cable Ladder 90 450</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>19f22aef-af24-3a1c-b63f-1703e94e50ba</t>
+          <t>167265d4-c3e5-3071-b189-599004f7b9f3</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1JNL9442575_A-MVS Cable Ladder P1</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>76440f25-e447-3cc5-958e-8727a44d872d</t>
+          <t>366c5df3-80dd-34c1-95f6-f69c55125c61</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1JNL9442576_A-K6 cable tray MVS P1</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5b00d1af-e807-3f5e-bc90-b4ab1b39b423</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>9</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>c91648b7-3272-3ce6-92e1-f4279dbf9478</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1JNL9442631_A-Cable Ladder MVS</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>366c5df3-80dd-34c1-95f6-f69c55125c61</t>
+          <t>69eed907-29dc-3444-89dd-6e9fe484ce1b</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1JNL9442631_A-Cable Ladder MVS</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>69eed907-29dc-3444-89dd-6e9fe484ce1b</t>
+          <t>97558d3b-c88d-3c4c-b66f-b2109faa27c0</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1JNL9442631_A-Cable Ladder MVS</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>97558d3b-c88d-3c4c-b66f-b2109faa27c0</t>
+          <t>a378d9c0-1349-32e1-9dad-1b5310fafdc9</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1JNL9442632_A-Cable Ladder MVS</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -645,13 +645,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1JNL9442632_A-Cable Ladder MVS</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -663,13 +663,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1JNL9442632_A-Cable Ladder MVS</t>
+          <t>A-Cable Ladder MVS</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -681,61 +681,61 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1JNL9442633_A-Cable Ladder MVS</t>
+          <t>A-Electrical design requirements, MVS1, NER, Aux Tx-building, Cable ways</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>167265d4-c3e5-3071-b189-599004f7b9f3</t>
+          <t>cd06ec2a-dde8-35e7-bb84-94eaba646aaa</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1JNL9442633_A-Cable Ladder MVS</t>
+          <t>A-K6 cable tray MVS P1</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5b00d1af-e807-3f5e-bc90-b4ab1b39b423</t>
+          <t>c91648b7-3272-3ce6-92e1-f4279dbf9478</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1JNL9442633_A-Cable Ladder MVS</t>
+          <t>A-MVS Cable Ladder P1</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>a378d9c0-1349-32e1-9dad-1b5310fafdc9</t>
+          <t>76440f25-e447-3cc5-958e-8727a44d872d</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">

</xml_diff>